<commit_message>
Fix test-scenarios generator: add safety, prior insurance, fix data types
- Added 12 explicit safety features (Yes) to application template
- Added complete prior insurance details (carrier, policy, premium)
- Added driver breakdown (regular/part-time/owner-operators)
- Changed violations/accidents default from 'None' to 0
- Changed vehicle value default to $95,000 (full amount)
- Regenerated all 5 test scenarios
</commit_message>
<xml_diff>
--- a/sample-data/test-scenarios/test-1-perfect/Heartland_Express_Inc_Driver_Roster.xlsx
+++ b/sample-data/test-scenarios/test-1-perfect/Heartland_Express_Inc_Driver_Roster.xlsx
@@ -518,15 +518,11 @@
           <t>2020-01-15</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -574,15 +570,11 @@
           <t>2020-01-15</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -630,15 +622,11 @@
           <t>2020-01-15</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -686,15 +674,11 @@
           <t>2020-01-15</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -742,15 +726,11 @@
           <t>2020-01-15</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>

</xml_diff>